<commit_message>
feat: update the XSLT file to consider the grouper effectiveTime in observation resource id generation for CureMD CCDA files #3360 - update the CCDA to FHIR conversion specification document for CureMD.
</commit_message>
<xml_diff>
--- a/support/specifications/ccda/CCDA to FHIR Conversion Spec - CureMD.xlsx
+++ b/support/specifications/ccda/CCDA to FHIR Conversion Spec - CureMD.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="709" activeTab="1"/>
+    <workbookView windowWidth="19200" windowHeight="8000" tabRatio="709" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="CureMD" sheetId="11" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="457">
   <si>
     <t>Epic CCDA</t>
   </si>
@@ -295,6 +295,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>If there is an entry in the Social History section [code.code = '</t>
     </r>
     <r>
@@ -403,6 +410,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Document.component.structuredBody.component.section[code=</t>
     </r>
     <r>
@@ -454,6 +468,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Document.component.structuredBody.component.section[code.code = '</t>
     </r>
     <r>
@@ -1826,6 +1847,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">For </t>
     </r>
     <r>
@@ -2274,6 +2301,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">For </t>
     </r>
     <r>
@@ -3911,6 +3944,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">For </t>
     </r>
     <r>
@@ -3954,7 +3993,7 @@
   </si>
   <si>
     <t>Facility ID (from the header variable `X-TechBD-Facility-ID`) + '-' + question code (code.code) + '-' + id.extension value from the Observation element.
-If id.extension is not available then will use effectiveDateTime calculated of the observation resource.</t>
+If effectiveTime is not present in the observation, then use the grouper effectiveTime, if it is also not present then use encounter effectiveTime.</t>
   </si>
   <si>
     <t>"id": "ACPNY-88122-7-flo1572879820-5810220439-97051-Z549669"</t>
@@ -4525,9 +4564,14 @@
       },</t>
   </si>
   <si>
+    <t>effectiveTime.value OR 
+effectiveTime.low.value</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">First check the value from entryRelationship.observation.effectiveTime. 
-`Document.component.section.entry.observation.entryRelationship.observation.effectiveTime`
+`Document.component.section.entry.observation.entryRelationship.observation.effectiveTime.value`
+If effectiveTime is not present in the observation, then use the grouper effectiveTime.
 If that is not valued, then use the same timestamp that is used in the Encounter FHIR resource:
 for </t>
     </r>
@@ -4548,7 +4592,7 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>: Document.component.structuredBody.component.section[code.code='46240-8']/.entry[1].encounter.effectiveTime
+      <t>: Document.component.structuredBody.component.section[code.code='46240-8']/.entry[1].encounter.effectiveTime.value OR effectiveTime.low.value
 If that is not valued, then use the same timestamp that is used in the meta.lastUpdated.</t>
     </r>
   </si>
@@ -4568,6 +4612,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">For </t>
     </r>
     <r>
@@ -4624,26 +4674,6 @@
   </si>
   <si>
     <t>Provided the fixed value, "en"</t>
-  </si>
-  <si>
-    <r>
-      <t>statusCode.code -&gt; status Mapping</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-completed -&gt; final 
-final -&gt; final 
-aborted -&gt; entered-in-error  
-cancelled -&gt; entered-in-error  
-nullified -&gt; entered-in-error 
-All Others -&gt; unknown</t>
-    </r>
   </si>
   <si>
     <t>"category": [
@@ -4725,6 +4755,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">For </t>
     </r>
     <r>
@@ -5066,6 +5102,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>First check the value from entryRelationship.observation.effectiveTime. 
 for</t>
     </r>
@@ -5135,6 +5177,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">For </t>
     </r>
     <r>
@@ -5500,16 +5548,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <i/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5977,7 +6025,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6066,9 +6114,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -6620,20 +6665,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="8.88571428571429" style="32"/>
-    <col min="2" max="2" width="35.2190476190476" customWidth="1"/>
-    <col min="3" max="3" width="92.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="8.88181818181818" style="31"/>
+    <col min="2" max="2" width="35.2181818181818" customWidth="1"/>
+    <col min="3" max="3" width="92.6636363636364" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="32" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="32">
+      <c r="A3" s="31">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -6644,7 +6689,7 @@
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="32">
+      <c r="A4" s="31">
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -6655,7 +6700,7 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="32">
+      <c r="A5" s="31">
         <v>3</v>
       </c>
       <c r="B5" s="15" t="s">
@@ -6666,7 +6711,7 @@
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="32">
+      <c r="A6" s="31">
         <v>4</v>
       </c>
       <c r="B6" s="24" t="s">
@@ -6677,10 +6722,10 @@
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="32">
+      <c r="A7" s="31">
         <v>5</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="33" t="s">
         <v>3</v>
       </c>
       <c r="C7" t="s">
@@ -6697,14 +6742,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.5727272727273" customWidth="1"/>
     <col min="3" max="3" width="53" customWidth="1"/>
-    <col min="4" max="4" width="72.2857142857143" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="47.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="72.2818181818182" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="47.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -6747,7 +6792,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="4" ht="120" spans="1:6">
+    <row r="4" ht="116" spans="1:6">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -6770,7 +6815,7 @@
       <c r="D5"/>
       <c r="E5" s="6"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
@@ -6798,7 +6843,7 @@
       <c r="E7" s="11"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" ht="75" spans="1:6">
+    <row r="8" ht="72.5" spans="1:6">
       <c r="B8" s="4" t="s">
         <v>85</v>
       </c>
@@ -6812,7 +6857,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="9" ht="60" spans="1:6">
+    <row r="9" ht="58" spans="1:6">
       <c r="B9" s="4" t="s">
         <v>89</v>
       </c>
@@ -6938,14 +6983,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="28.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="65.4571428571429" customWidth="1"/>
-    <col min="4" max="4" width="46.2190476190476" customWidth="1"/>
-    <col min="5" max="5" width="61.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="46.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="28.3363636363636" customWidth="1"/>
+    <col min="3" max="3" width="65.4545454545455" customWidth="1"/>
+    <col min="4" max="4" width="46.2181818181818" customWidth="1"/>
+    <col min="5" max="5" width="61.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="46.2818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -7043,7 +7088,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" ht="30" spans="1:6">
+    <row r="10" ht="29" spans="1:6">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -7064,7 +7109,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" ht="45" spans="2:7">
+    <row r="17" ht="43.5" spans="2:7">
       <c r="B17" t="s">
         <v>35</v>
       </c>
@@ -7080,7 +7125,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" ht="150" spans="2:7">
+    <row r="19" ht="116" spans="2:7">
       <c r="B19" t="s">
         <v>39</v>
       </c>
@@ -7089,7 +7134,7 @@
       </c>
       <c r="E19" s="29"/>
     </row>
-    <row r="20" ht="45" spans="2:7">
+    <row r="20" ht="29" spans="2:7">
       <c r="B20" s="4" t="s">
         <v>41</v>
       </c>
@@ -7098,7 +7143,7 @@
       </c>
       <c r="E20" s="10"/>
     </row>
-    <row r="21" ht="45" spans="2:7">
+    <row r="21" ht="43.5" spans="2:7">
       <c r="B21" t="s">
         <v>43</v>
       </c>
@@ -7107,17 +7152,17 @@
       </c>
       <c r="E21" s="10"/>
     </row>
-    <row r="22" ht="30" spans="2:7">
+    <row r="22" ht="29" spans="2:7">
       <c r="B22" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="10" t="s">
         <v>46</v>
       </c>
       <c r="E22" s="6"/>
     </row>
-    <row r="23" ht="45" spans="2:7">
-      <c r="B23" s="31" t="s">
+    <row r="23" ht="43.5" spans="2:7">
+      <c r="B23" s="30" t="s">
         <v>47</v>
       </c>
       <c r="C23" s="10" t="s">
@@ -7144,13 +7189,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="41.7809523809524" style="4" customWidth="1"/>
-    <col min="3" max="3" width="65.0952380952381" style="4" customWidth="1"/>
-    <col min="4" max="4" width="81.2857142857143" style="4" customWidth="1"/>
-    <col min="5" max="5" width="48.4285714285714" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="41.7818181818182" style="4" customWidth="1"/>
+    <col min="3" max="3" width="65.0909090909091" style="4" customWidth="1"/>
+    <col min="4" max="4" width="81.2818181818182" style="4" customWidth="1"/>
+    <col min="5" max="5" width="48.4272727272727" style="4" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7188,7 +7233,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" ht="90" spans="1:6">
+    <row r="4" ht="87" spans="1:6">
       <c r="B4" s="17" t="s">
         <v>16</v>
       </c>
@@ -7216,7 +7261,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" ht="30" spans="1:6">
+    <row r="7" ht="29" spans="1:6">
       <c r="B7" s="4" t="s">
         <v>56</v>
       </c>
@@ -7227,7 +7272,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" ht="60" spans="1:6">
+    <row r="8" ht="58" spans="1:6">
       <c r="B8" s="4" t="s">
         <v>59</v>
       </c>
@@ -7283,7 +7328,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" ht="60" spans="1:6">
+    <row r="13" ht="58" spans="1:6">
       <c r="B13" s="4" t="s">
         <v>73</v>
       </c>
@@ -7294,7 +7339,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="1:6">
+    <row r="14" ht="29" spans="1:6">
       <c r="B14" s="4" t="s">
         <v>76</v>
       </c>
@@ -7305,7 +7350,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" ht="30" spans="1:6">
+    <row r="15" spans="1:6">
       <c r="B15" s="4" t="s">
         <v>79</v>
       </c>
@@ -7327,7 +7372,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="17" ht="75" spans="2:5">
+    <row r="17" ht="72.5" spans="2:5">
       <c r="B17" s="4" t="s">
         <v>85</v>
       </c>
@@ -7341,7 +7386,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="18" ht="60" spans="2:5">
+    <row r="18" ht="58" spans="2:5">
       <c r="B18" s="4" t="s">
         <v>89</v>
       </c>
@@ -7395,7 +7440,7 @@
       </c>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" ht="120" spans="2:5">
+    <row r="24" ht="116" spans="2:5">
       <c r="B24" s="4" t="s">
         <v>101</v>
       </c>
@@ -7414,7 +7459,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="26" ht="90" spans="2:5">
+    <row r="26" ht="87" spans="2:5">
       <c r="B26" s="4" t="s">
         <v>106</v>
       </c>
@@ -7425,7 +7470,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="27" ht="45" spans="2:5">
+    <row r="27" ht="43.5" spans="2:5">
       <c r="B27" s="4" t="s">
         <v>109</v>
       </c>
@@ -7439,7 +7484,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="28" ht="30" spans="2:5">
+    <row r="28" spans="2:5">
       <c r="B28" s="4" t="s">
         <v>113</v>
       </c>
@@ -7459,7 +7504,7 @@
       <c r="D29" s="14"/>
       <c r="E29" s="6"/>
     </row>
-    <row r="30" ht="30" spans="2:5">
+    <row r="30" spans="2:5">
       <c r="B30" s="4" t="s">
         <v>117</v>
       </c>
@@ -7479,7 +7524,7 @@
       <c r="D31" s="14"/>
       <c r="E31" s="6"/>
     </row>
-    <row r="32" ht="45" spans="2:5">
+    <row r="32" ht="43.5" spans="2:5">
       <c r="B32" s="4" t="s">
         <v>109</v>
       </c>
@@ -7493,7 +7538,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="33" ht="30" spans="2:6">
+    <row r="33" spans="2:6">
       <c r="B33" s="4" t="s">
         <v>113</v>
       </c>
@@ -7511,7 +7556,7 @@
       </c>
       <c r="D34" s="14"/>
     </row>
-    <row r="35" ht="30" spans="2:6">
+    <row r="35" spans="2:6">
       <c r="B35" s="4" t="s">
         <v>117</v>
       </c>
@@ -7540,7 +7585,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="38" ht="45" spans="2:6">
+    <row r="38" ht="43.5" spans="2:6">
       <c r="B38" s="4" t="s">
         <v>129</v>
       </c>
@@ -7548,11 +7593,11 @@
         <v>80</v>
       </c>
       <c r="D38" s="14"/>
-      <c r="E38" s="35" t="s">
+      <c r="E38" s="34" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="39" ht="120" spans="2:6">
+    <row r="39" ht="116" spans="2:6">
       <c r="B39" s="4" t="s">
         <v>131</v>
       </c>
@@ -7563,7 +7608,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="40" ht="120" spans="2:6">
+    <row r="40" ht="116" spans="2:6">
       <c r="B40" s="4" t="s">
         <v>134</v>
       </c>
@@ -7610,7 +7655,7 @@
       </c>
       <c r="D44" s="10"/>
     </row>
-    <row r="45" ht="195" spans="2:6">
+    <row r="45" ht="188.5" spans="2:6">
       <c r="B45" s="17" t="s">
         <v>144</v>
       </c>
@@ -7624,7 +7669,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="46" ht="195" spans="2:6">
+    <row r="46" ht="188.5" spans="2:6">
       <c r="B46" s="17" t="s">
         <v>148</v>
       </c>
@@ -7638,7 +7683,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="47" ht="195" spans="2:6">
+    <row r="47" ht="188.5" spans="2:6">
       <c r="B47" s="17" t="s">
         <v>152</v>
       </c>
@@ -7690,7 +7735,7 @@
       <c r="D51" s="10"/>
       <c r="E51" s="4"/>
     </row>
-    <row r="52" ht="150" spans="2:6">
+    <row r="52" ht="145" spans="2:6">
       <c r="B52" s="10" t="s">
         <v>161</v>
       </c>
@@ -7764,7 +7809,7 @@
       <c r="D58" s="10"/>
       <c r="E58" s="6"/>
     </row>
-    <row r="59" ht="180" spans="2:6">
+    <row r="59" ht="174" spans="2:6">
       <c r="B59" s="10" t="s">
         <v>175</v>
       </c>
@@ -7778,7 +7823,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="60" ht="255" spans="2:6">
+    <row r="60" ht="246.5" spans="2:6">
       <c r="B60" s="4" t="s">
         <v>178</v>
       </c>
@@ -7789,7 +7834,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="61" ht="45" spans="2:6">
+    <row r="61" ht="43.5" spans="2:6">
       <c r="B61" s="4" t="s">
         <v>181</v>
       </c>
@@ -7809,7 +7854,7 @@
       <c r="D62" s="10"/>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" ht="210" spans="2:6">
+    <row r="63" ht="203" spans="2:6">
       <c r="B63" s="4" t="s">
         <v>185</v>
       </c>
@@ -7887,14 +7932,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="30.8571428571429" customWidth="1"/>
-    <col min="3" max="3" width="63.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="70.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="52.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="57.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="30.8545454545455" customWidth="1"/>
+    <col min="3" max="3" width="63.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="70.7181818181818" customWidth="1"/>
+    <col min="5" max="5" width="52.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="57.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:7">
@@ -7936,7 +7981,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="4" ht="105" spans="1:7">
+    <row r="4" ht="101.5" spans="1:7">
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
@@ -7968,7 +8013,7 @@
       </c>
       <c r="E6" s="24"/>
     </row>
-    <row r="7" ht="120" spans="1:7">
+    <row r="7" ht="116" spans="1:7">
       <c r="B7" s="5" t="s">
         <v>203</v>
       </c>
@@ -8021,7 +8066,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="11" ht="225" spans="1:7">
+    <row r="11" ht="203" spans="1:7">
       <c r="B11" s="5" t="s">
         <v>215</v>
       </c>
@@ -8057,7 +8102,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="1:7">
+    <row r="14" ht="29" spans="1:7">
       <c r="B14" s="5" t="s">
         <v>222</v>
       </c>
@@ -8071,7 +8116,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="15" ht="45" spans="1:7">
+    <row r="15" ht="43.5" spans="1:7">
       <c r="B15" s="5" t="s">
         <v>226</v>
       </c>
@@ -8085,7 +8130,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="16" ht="45" spans="1:7">
+    <row r="16" ht="43.5" spans="1:7">
       <c r="B16" s="5" t="s">
         <v>230</v>
       </c>
@@ -8097,7 +8142,7 @@
       </c>
       <c r="E16" s="6"/>
     </row>
-    <row r="17" ht="45" spans="2:6">
+    <row r="17" ht="43.5" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>233</v>
       </c>
@@ -8109,7 +8154,7 @@
       </c>
       <c r="E17" s="6"/>
     </row>
-    <row r="18" ht="45" spans="2:6">
+    <row r="18" ht="43.5" spans="2:6">
       <c r="B18" t="s">
         <v>236</v>
       </c>
@@ -8123,7 +8168,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="19" ht="60" spans="2:6">
+    <row r="19" ht="58" spans="2:6">
       <c r="B19" s="5" t="s">
         <v>239</v>
       </c>
@@ -8188,14 +8233,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="35.1428571428571" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="35.1454545454545" customWidth="1"/>
     <col min="3" max="3" width="53" style="4" customWidth="1"/>
-    <col min="4" max="4" width="73.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="73.5727272727273" customWidth="1"/>
     <col min="5" max="5" width="53" customWidth="1"/>
-    <col min="6" max="6" width="51.7142857142857" customWidth="1"/>
+    <col min="6" max="6" width="51.7181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8237,7 +8282,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="4" ht="165" spans="1:6">
+    <row r="4" ht="159.5" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -8262,7 +8307,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="17" t="s">
         <v>22</v>
       </c>
@@ -8273,7 +8318,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" ht="165" spans="1:6">
+    <row r="7" ht="159.5" spans="1:6">
       <c r="B7" s="5" t="s">
         <v>203</v>
       </c>
@@ -8330,7 +8375,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="12" ht="60" spans="1:6">
+    <row r="12" ht="58" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>264</v>
       </c>
@@ -8356,7 +8401,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="15" customFormat="1" ht="60" spans="1:6">
+    <row r="15" customFormat="1" ht="58" spans="1:6">
       <c r="B15" s="5" t="s">
         <v>270</v>
       </c>
@@ -8367,7 +8412,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="16" customFormat="1" ht="30" spans="1:6">
+    <row r="16" customFormat="1" spans="1:6">
       <c r="B16" s="5" t="s">
         <v>272</v>
       </c>
@@ -8375,7 +8420,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="17" ht="60" spans="2:5">
+    <row r="17" ht="58" spans="2:5">
       <c r="B17" t="s">
         <v>274</v>
       </c>
@@ -8394,7 +8439,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="19" ht="45" spans="2:5">
+    <row r="19" ht="43.5" spans="2:5">
       <c r="B19" t="s">
         <v>279</v>
       </c>
@@ -8417,7 +8462,7 @@
       </c>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" ht="105" spans="2:5">
+    <row r="21" ht="101.5" spans="2:5">
       <c r="B21" t="s">
         <v>285</v>
       </c>
@@ -8428,7 +8473,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="22" ht="60" spans="2:5">
+    <row r="22" ht="58" spans="2:5">
       <c r="B22" t="s">
         <v>288</v>
       </c>
@@ -8497,14 +8542,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="27.3333333333333" customWidth="1"/>
-    <col min="3" max="3" width="50.8857142857143" customWidth="1"/>
-    <col min="4" max="4" width="72.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="46.4285714285714" customWidth="1"/>
-    <col min="6" max="6" width="45.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="27.3363636363636" customWidth="1"/>
+    <col min="3" max="3" width="50.8818181818182" customWidth="1"/>
+    <col min="4" max="4" width="72.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="46.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="45.7181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -8540,7 +8585,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="4" ht="135" spans="1:6">
+    <row r="4" ht="130.5" spans="1:6">
       <c r="B4" t="s">
         <v>16</v>
       </c>
@@ -8565,7 +8610,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
@@ -8614,7 +8659,7 @@
       <c r="D9" s="10"/>
       <c r="E9" s="6"/>
     </row>
-    <row r="10" ht="30" spans="1:6">
+    <row r="10" ht="29" spans="1:6">
       <c r="B10" s="4" t="s">
         <v>312</v>
       </c>
@@ -8624,7 +8669,7 @@
       <c r="D10" s="10"/>
       <c r="E10" s="6"/>
     </row>
-    <row r="11" ht="30" spans="1:6">
+    <row r="11" ht="29" spans="1:6">
       <c r="B11" s="4" t="s">
         <v>314</v>
       </c>
@@ -8634,7 +8679,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="6"/>
     </row>
-    <row r="12" ht="30" spans="1:6">
+    <row r="12" ht="29" spans="1:6">
       <c r="B12" s="4" t="s">
         <v>315</v>
       </c>
@@ -8668,7 +8713,7 @@
       <c r="D14" s="10"/>
       <c r="E14" s="20"/>
     </row>
-    <row r="15" customFormat="1" ht="30" spans="1:6">
+    <row r="15" customFormat="1" ht="29" spans="1:6">
       <c r="B15" s="4" t="s">
         <v>322</v>
       </c>
@@ -8678,7 +8723,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="20"/>
     </row>
-    <row r="16" customFormat="1" ht="30" spans="1:6">
+    <row r="16" customFormat="1" ht="29" spans="1:6">
       <c r="B16" s="4" t="s">
         <v>324</v>
       </c>
@@ -8688,7 +8733,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="1" ht="30" spans="2:6">
+    <row r="17" customFormat="1" ht="29" spans="2:6">
       <c r="B17" s="4" t="s">
         <v>325</v>
       </c>
@@ -8697,7 +8742,7 @@
       </c>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" ht="60" spans="2:6">
+    <row r="18" ht="58" spans="2:6">
       <c r="B18" s="5" t="s">
         <v>327</v>
       </c>
@@ -8732,7 +8777,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="21" customFormat="1" ht="120" spans="2:6">
+    <row r="21" customFormat="1" ht="116" spans="2:6">
       <c r="B21" s="4" t="s">
         <v>101</v>
       </c>
@@ -8745,7 +8790,7 @@
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" customFormat="1" ht="30" spans="2:6">
+    <row r="22" customFormat="1" ht="29" spans="2:6">
       <c r="B22" s="4" t="s">
         <v>104</v>
       </c>
@@ -8755,7 +8800,7 @@
       <c r="D22" s="10"/>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" customFormat="1" ht="90" spans="2:6">
+    <row r="23" customFormat="1" ht="87" spans="2:6">
       <c r="B23" s="4" t="s">
         <v>106</v>
       </c>
@@ -8768,7 +8813,7 @@
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" customFormat="1" ht="120" spans="2:6">
+    <row r="24" customFormat="1" ht="116" spans="2:6">
       <c r="B24" s="4" t="s">
         <v>89</v>
       </c>
@@ -8781,7 +8826,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" customFormat="1" ht="75" spans="2:6">
+    <row r="25" customFormat="1" ht="72.5" spans="2:6">
       <c r="B25" s="4" t="s">
         <v>85</v>
       </c>
@@ -8794,7 +8839,7 @@
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" customFormat="1" ht="30" spans="2:6">
+    <row r="26" customFormat="1" ht="29" spans="2:6">
       <c r="B26" s="4" t="s">
         <v>91</v>
       </c>
@@ -8805,7 +8850,7 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" customFormat="1" ht="30" spans="2:6">
+    <row r="27" customFormat="1" ht="29" spans="2:6">
       <c r="B27" s="4" t="s">
         <v>93</v>
       </c>
@@ -8816,7 +8861,7 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" customFormat="1" ht="30" spans="2:6">
+    <row r="28" customFormat="1" ht="29" spans="2:6">
       <c r="B28" s="4" t="s">
         <v>95</v>
       </c>
@@ -8827,7 +8872,7 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" customFormat="1" ht="30" spans="2:6">
+    <row r="29" customFormat="1" ht="29" spans="2:6">
       <c r="B29" s="4" t="s">
         <v>97</v>
       </c>
@@ -8838,7 +8883,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" customFormat="1" ht="30" spans="2:6">
+    <row r="30" customFormat="1" ht="29" spans="2:6">
       <c r="B30" s="4" t="s">
         <v>99</v>
       </c>
@@ -8887,13 +8932,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.88181818181818" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.8857142857143" customWidth="1"/>
-    <col min="3" max="3" width="58.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="57.1142857142857" customWidth="1"/>
-    <col min="5" max="5" width="54.7142857142857" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.8818181818182" customWidth="1"/>
+    <col min="3" max="3" width="58.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="57.1181818181818" customWidth="1"/>
+    <col min="5" max="5" width="54.7181818181818" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8917,7 +8962,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" ht="45" spans="1:6">
+    <row r="2" ht="43.5" spans="1:6">
       <c r="A2" s="19" t="s">
         <v>351</v>
       </c>
@@ -8931,7 +8976,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="4" ht="255" spans="1:6">
+    <row r="4" ht="232" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -8955,7 +9000,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" ht="30" spans="1:6">
+    <row r="6" ht="29" spans="1:6">
       <c r="B6" s="17" t="s">
         <v>22</v>
       </c>
@@ -8977,7 +9022,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="8" ht="150" spans="1:6">
+    <row r="8" ht="145" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>203</v>
       </c>
@@ -9002,7 +9047,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="10" ht="30" spans="1:6">
+    <row r="10" ht="29" spans="1:6">
       <c r="B10" s="5" t="s">
         <v>363</v>
       </c>
@@ -9021,7 +9066,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="6"/>
     </row>
-    <row r="12" ht="30" spans="1:6">
+    <row r="12" ht="29" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>366</v>
       </c>
@@ -9041,7 +9086,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="14" ht="30" spans="1:6">
+    <row r="14" ht="29" spans="1:6">
       <c r="B14" s="4" t="s">
         <v>370</v>
       </c>
@@ -9062,7 +9107,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="16" ht="75" spans="1:6">
+    <row r="16" ht="58" spans="1:6">
       <c r="B16" s="5" t="s">
         <v>270</v>
       </c>
@@ -9081,7 +9126,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="18" ht="90" spans="2:6">
+    <row r="18" ht="87" spans="2:6">
       <c r="B18" t="s">
         <v>375</v>
       </c>
@@ -9141,14 +9186,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="34.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="49.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="58.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="50.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="34.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="49.6636363636364" customWidth="1"/>
+    <col min="4" max="4" width="58.7181818181818" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="50.2818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9192,7 +9237,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="4" ht="90" spans="1:6">
+    <row r="4" ht="87" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
@@ -9216,7 +9261,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="17" t="s">
         <v>22</v>
       </c>
@@ -9238,7 +9283,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="8" ht="105" spans="1:6">
+    <row r="8" ht="101.5" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>203</v>
       </c>
@@ -9263,7 +9308,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="10" ht="45" spans="1:6">
+    <row r="10" ht="43.5" spans="1:6">
       <c r="B10" s="5" t="s">
         <v>220</v>
       </c>
@@ -9275,7 +9320,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="11" ht="210" spans="1:6">
+    <row r="11" ht="203" spans="1:6">
       <c r="B11" s="5" t="s">
         <v>215</v>
       </c>
@@ -9284,7 +9329,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="12" ht="210" spans="1:6">
+    <row r="12" ht="203" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>218</v>
       </c>
@@ -9334,7 +9379,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="9"/>
     </row>
-    <row r="17" ht="30" spans="2:6">
+    <row r="17" ht="29" spans="2:6">
       <c r="B17" s="5" t="s">
         <v>366</v>
       </c>
@@ -9346,7 +9391,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="18" ht="105" spans="2:6">
+    <row r="18" ht="101.5" spans="2:6">
       <c r="B18" s="4" t="s">
         <v>367</v>
       </c>
@@ -9360,7 +9405,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="19" ht="30" spans="2:6">
+    <row r="19" ht="29" spans="2:6">
       <c r="B19" s="4" t="s">
         <v>370</v>
       </c>
@@ -9368,7 +9413,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="20" ht="30" spans="2:6">
+    <row r="20" ht="29" spans="2:6">
       <c r="B20" s="4" t="s">
         <v>372</v>
       </c>
@@ -9388,7 +9433,7 @@
       </c>
       <c r="E21" s="6"/>
     </row>
-    <row r="22" ht="75" spans="2:6">
+    <row r="22" ht="72.5" spans="2:6">
       <c r="B22" s="5" t="s">
         <v>409</v>
       </c>
@@ -9400,7 +9445,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="23" ht="45" spans="2:6">
+    <row r="23" ht="43.5" spans="2:6">
       <c r="B23" s="5" t="s">
         <v>412</v>
       </c>
@@ -9409,7 +9454,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="24" ht="60" spans="2:6">
+    <row r="24" ht="58" spans="2:6">
       <c r="B24" s="5" t="s">
         <v>270</v>
       </c>
@@ -9420,7 +9465,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="25" ht="30" spans="2:6">
+    <row r="25" ht="29" spans="2:6">
       <c r="B25" s="5" t="s">
         <v>272</v>
       </c>
@@ -9428,7 +9473,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="26" ht="45" spans="2:6">
+    <row r="26" ht="43.5" spans="2:6">
       <c r="B26" s="5" t="s">
         <v>414</v>
       </c>
@@ -9439,27 +9484,29 @@
         <v>416</v>
       </c>
     </row>
-    <row r="27" ht="195" spans="2:6">
+    <row r="27" ht="246.5" spans="2:6">
       <c r="B27" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="4" t="s">
+        <v>417</v>
+      </c>
       <c r="D27" t="s">
         <v>377</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="28" ht="45" spans="2:6">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="28" ht="43.5" spans="2:6">
       <c r="B28" s="5" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>234</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="29" spans="2:6">
@@ -9482,7 +9529,7 @@
         <v>194</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="31" ht="46" customHeight="1" spans="2:6">
@@ -9511,14 +9558,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="63.1428571428571" customWidth="1"/>
-    <col min="4" max="4" width="56.552380952381" customWidth="1"/>
-    <col min="5" max="5" width="53.2857142857143" customWidth="1"/>
-    <col min="6" max="6" width="47.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="14.7181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="63.1454545454545" customWidth="1"/>
+    <col min="4" max="4" width="56.5545454545455" customWidth="1"/>
+    <col min="5" max="5" width="53.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="47.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -9546,7 +9593,7 @@
         <v>43</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -9562,16 +9609,16 @@
         <v>352</v>
       </c>
     </row>
-    <row r="4" ht="180" spans="1:6">
+    <row r="4" ht="174" spans="1:6">
       <c r="A4" s="1"/>
       <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D4" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="5" customFormat="1" spans="1:6">
@@ -9586,7 +9633,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="1" ht="30" spans="1:6">
+    <row r="6" customFormat="1" ht="29" spans="1:6">
       <c r="B6" s="17" t="s">
         <v>22</v>
       </c>
@@ -9605,13 +9652,13 @@
         <v>58</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="8" ht="105" spans="1:6">
+    <row r="8" ht="101.5" spans="1:6">
       <c r="B8" s="5" t="s">
         <v>203</v>
       </c>
@@ -9622,7 +9669,7 @@
         <v>358</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>425</v>
+        <v>389</v>
       </c>
     </row>
     <row r="9" ht="409" customHeight="1" spans="1:6">
@@ -9636,7 +9683,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="10" ht="240" spans="1:6">
+    <row r="10" ht="232" spans="1:6">
       <c r="B10" s="5" t="s">
         <v>360</v>
       </c>
@@ -9650,7 +9697,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="11" ht="180" spans="1:6">
+    <row r="11" ht="159.5" spans="1:6">
       <c r="B11" s="5" t="s">
         <v>363</v>
       </c>
@@ -9659,7 +9706,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="12" ht="150" spans="1:6">
+    <row r="12" ht="145" spans="1:6">
       <c r="B12" s="5" t="s">
         <v>365</v>
       </c>
@@ -9668,7 +9715,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="13" ht="75" spans="1:6">
+    <row r="13" ht="58" spans="1:6">
       <c r="B13" s="5" t="s">
         <v>270</v>
       </c>
@@ -9687,7 +9734,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="15" ht="45" spans="1:6">
+    <row r="15" ht="43.5" spans="1:6">
       <c r="B15" s="5" t="s">
         <v>414</v>
       </c>
@@ -9698,7 +9745,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="16" ht="210" spans="1:6">
+    <row r="16" ht="203" spans="1:6">
       <c r="B16" s="5" t="s">
         <v>375</v>
       </c>
@@ -9710,15 +9757,15 @@
         <v>432</v>
       </c>
     </row>
-    <row r="17" ht="45" spans="2:6">
+    <row r="17" ht="43.5" spans="2:6">
       <c r="B17" s="5" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>234</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="18" spans="2:6">
@@ -9735,7 +9782,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="19" ht="165" spans="2:6">
+    <row r="19" ht="159.5" spans="2:6">
       <c r="B19" t="s">
         <v>434</v>
       </c>
@@ -9754,7 +9801,7 @@
         <v>194</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1" spans="2:6">

</xml_diff>